<commit_message>
Adicionado mais 3 empresas
</commit_message>
<xml_diff>
--- a/enviando/empresas_descricoes.xlsx
+++ b/enviando/empresas_descricoes.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -872,7 +872,7 @@
     <row r="17" ht="120" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>sao-jose-viagens</t>
+          <t>brasil-way-tour</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1465,7 +1465,7 @@
     <row r="39" ht="120" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>viacao-nova</t>
+          <t>expresso-adamantina</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -1731,6 +1731,72 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>gimenes-turismo</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Gimenes Turismo</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Com mais de 40 anos de atuação, a Gimenes Turismo é uma empresa familiar que se destaca pela confiabilidade e qualidade em fretamento para viagens, com foco especial em São Paulo, oferecendo serviços de bate e volta para compras e negócios. Autorizada pela ANTT, a Gimenes prioriza a segurança e o conforto de seus passageiros.&lt;br&gt;&lt;br&gt;A frota da empresa é moderna e conta com ônibus equipados para garantir uma viagem agradável, incluindo poltronas reclináveis, ar-condicionado e Wi-Fi a bordo.&lt;br&gt;&lt;br&gt;Ao escolher a Gimenes, você pode reservar suas viagens de maneira prática e segura por meio da Buser, que proporciona um processo 100% digital, combinando tradição e inovação.</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Reserve sua viagem de ônibus com a Gimenes Turismo na Buser e aproveite toda a comodidade que você merece.&lt;br&gt;&lt;br&gt;A Gimenes Turismo é uma empresa familiar que se destaca no fretamento de ônibus para excursões, eventos e viagens em grupo. Ela também oferece transporte de encomendas entre São Paulo e Franca.&lt;br&gt;&lt;br&gt;Ao realizar sua reserva pela Buser, você tem à disposição um atendimento 24 horas, viagens seguras e poltronas confortáveis, proporcionando o máximo de conforto e tranquilidade durante o seu trajeto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>bompani-turismo</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Bompani Turismo</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Fundada em 2013, a Bompani Turismo é uma empresa de fretamento rodoviário situada em Luiz Alves, Santa Catarina. Com um forte foco em agenciamento de viagens, a empresa opera com a autorização da ANTT, o que assegura qualidade e segurança em suas operações.&lt;br&gt;&lt;br&gt;A Bompani se especializa em oferecer viagens personalizadas e excursões de turismo, conectando uma variedade de cidades e destinos. Um de seus grandes diferenciais é o conforto, que a destaca na realização de roteiros turísticos tanto regionais quanto internacionais.&lt;br&gt;&lt;br&gt;Sua frota é composta por veículos bem equipados, que oferecem comodidades como ar-condicionado e poltronas reclináveis, garantindo uma experiência agradável ao longo da viagem.&lt;br&gt;&lt;br&gt;Para reservar sua viagem com a Bompani, você pode usar a Buser, que proporciona um processo totalmente digital e seguro para reservar fretamentos de maneira prática e eficiente.</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Reserve sua viagem com a Bompani Turismo diretamente pela Buser, garantindo praticidade e confiança em cada etapa.&lt;br&gt;&lt;br&gt;A Bompani Turismo é especializada em fretamento de ônibus para turismo, oferecendo roteiros regionais, excursões e viagens de compras com todo o conforto e segurança que você merece.&lt;br&gt;&lt;br&gt;Ao reservar sua viagem de ônibus com a Bompani Turismo na Buser, você tem à disposição atendimento 24 horas, um trajeto seguro e a possibilidade de cancelamento grátis, tornando sua experiência ainda mais tranquila.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>jacson-turismo</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Jacson Turismo</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Fundada em Chapecó, Santa Catarina, a Jacson Turismo é uma empresa bem estabelecida no setor de transporte rodoviário, com autorização da ANTT para realizar fretamentos interestaduais.&lt;br&gt;&lt;br&gt;A companhia se destaca por oferecer viagens regulares direcionadas a lojistas e compradores, interligando cidades como São Paulo, Brusque e Criciúma, com saídas programadas em dias específicos da semana.&lt;br&gt;&lt;br&gt;Sua frota é composta por ônibus leito, que proporcionam conforto e comodidade ao longo das viagens, além de contar com serviços como café da manhã e suporte para o transporte de mercadorias.&lt;br&gt;&lt;br&gt;As viagens podem ser reservadas de maneira prática e segura por meio da Buser, uma parceria que combina a tradição da Jacson Turismo com a conveniência do processo digital.</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Garanta a sua viagem com a Jacson Turismo através da Buser, aproveitando toda a praticidade que você deseja.&lt;br&gt;&lt;br&gt;A Jacson Turismo é uma empresa de transporte rodoviário focada em fretamento, com roteiros que levam você a polos atacadistas, como São Paulo, Brusque e Criciúma.&lt;br&gt;&lt;br&gt;Ao reservar sua viagem de ônibus com a Jacson Turismo na Buser, você conta com atendimento 24 horas, poltronas confortáveis e um processo de reserva online simples, tornando sua experiência ainda mais agradável.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>